<commit_message>
resolve conflict from ML-Entrees 57e36e7983ba3d4528e00f2c44491168b6466bc8
</commit_message>
<xml_diff>
--- a/modeleLogiqueSBM/ig/StructureDefinition-fr-lm-allergy-intolerance.xlsx
+++ b/modeleLogiqueSBM/ig/StructureDefinition-fr-lm-allergy-intolerance.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="203">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-07T14:45:49+00:00</t>
+    <t>2026-04-08T10:07:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -406,15 +406,6 @@
   </si>
   <si>
     <t>fr-lm-entry.header.langue</t>
-  </si>
-  <si>
-    <t>fr-lm-allergy-intolerance.header.code</t>
-  </si>
-  <si>
-    <t>Type de l'entrée</t>
-  </si>
-  <si>
-    <t>fr-lm-entry.header.code</t>
   </si>
   <si>
     <t>fr-lm-allergy-intolerance.type</t>
@@ -960,7 +951,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ41"/>
+  <dimension ref="A1:AJ40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="49.61328125" customWidth="true" bestFit="true"/>
@@ -2523,7 +2514,7 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G16" t="s" s="2">
         <v>79</v>
@@ -2574,10 +2565,10 @@
         <v>73</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>73</v>
@@ -2595,10 +2586,10 @@
         <v>73</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AG16" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH16" t="s" s="2">
         <v>79</v>
@@ -2612,10 +2603,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2641,10 +2632,10 @@
         <v>121</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2674,10 +2665,10 @@
         <v>73</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>132</v>
+        <v>73</v>
       </c>
       <c r="Z17" t="s" s="2">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>73</v>
@@ -2695,7 +2686,7 @@
         <v>73</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -2712,10 +2703,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2741,10 +2732,10 @@
         <v>121</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2795,7 +2786,7 @@
         <v>73</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>79</v>
@@ -2812,10 +2803,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2823,7 +2814,7 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>79</v>
@@ -2838,7 +2829,7 @@
         <v>73</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="L19" t="s" s="2">
         <v>137</v>
@@ -2895,10 +2886,10 @@
         <v>73</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AG19" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH19" t="s" s="2">
         <v>79</v>
@@ -2938,13 +2929,13 @@
         <v>73</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="L20" t="s" s="2">
-        <v>140</v>
-      </c>
       <c r="M20" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2974,10 +2965,10 @@
         <v>73</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>73</v>
+        <v>140</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>73</v>
@@ -3012,10 +3003,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3041,10 +3032,10 @@
         <v>121</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3074,10 +3065,10 @@
         <v>73</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>73</v>
@@ -3095,7 +3086,7 @@
         <v>73</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>74</v>
@@ -3112,10 +3103,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3141,10 +3132,10 @@
         <v>121</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3174,10 +3165,10 @@
         <v>73</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>73</v>
@@ -3195,7 +3186,7 @@
         <v>73</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>74</v>
@@ -3212,10 +3203,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3223,7 +3214,7 @@
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>79</v>
@@ -3238,13 +3229,13 @@
         <v>73</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3274,10 +3265,10 @@
         <v>73</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>151</v>
+        <v>73</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>152</v>
+        <v>73</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>73</v>
@@ -3295,10 +3286,10 @@
         <v>73</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH23" t="s" s="2">
         <v>79</v>
@@ -3307,15 +3298,15 @@
         <v>73</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3323,7 +3314,7 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>79</v>
@@ -3338,13 +3329,13 @@
         <v>73</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="L24" t="s" s="2">
         <v>155</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3395,10 +3386,10 @@
         <v>73</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>79</v>
@@ -3407,26 +3398,26 @@
         <v>73</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>73</v>
@@ -3438,15 +3429,17 @@
         <v>73</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>163</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>73</v>
@@ -3483,50 +3476,50 @@
         <v>73</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>162</v>
+        <v>73</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>73</v>
@@ -3538,16 +3531,16 @@
         <v>73</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -3585,39 +3578,39 @@
         <v>73</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>167</v>
+        <v>73</v>
       </c>
       <c r="AC26" t="s" s="2">
-        <v>168</v>
+        <v>73</v>
       </c>
       <c r="AD26" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>169</v>
+        <v>73</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3625,7 +3618,7 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G27" t="s" s="2">
         <v>79</v>
@@ -3640,17 +3633,15 @@
         <v>73</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>175</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>73</v>
@@ -3699,10 +3690,10 @@
         <v>73</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AG27" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH27" t="s" s="2">
         <v>79</v>
@@ -3711,15 +3702,15 @@
         <v>73</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>73</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3742,13 +3733,13 @@
         <v>73</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>178</v>
+        <v>117</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3799,7 +3790,7 @@
         <v>73</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>74</v>
@@ -3811,15 +3802,15 @@
         <v>73</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>182</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3845,10 +3836,10 @@
         <v>117</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3899,7 +3890,7 @@
         <v>73</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>74</v>
@@ -3916,10 +3907,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -3930,7 +3921,7 @@
         <v>74</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>73</v>
@@ -3942,13 +3933,13 @@
         <v>73</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -3999,13 +3990,13 @@
         <v>73</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>73</v>
@@ -4016,10 +4007,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4030,7 +4021,7 @@
         <v>74</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>73</v>
@@ -4042,13 +4033,13 @@
         <v>73</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>80</v>
+        <v>121</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4078,7 +4069,7 @@
         <v>73</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>73</v>
+        <v>188</v>
       </c>
       <c r="Z31" t="s" s="2">
         <v>73</v>
@@ -4099,13 +4090,13 @@
         <v>73</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>73</v>
@@ -4127,7 +4118,7 @@
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G32" t="s" s="2">
         <v>79</v>
@@ -4202,7 +4193,7 @@
         <v>189</v>
       </c>
       <c r="AG32" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH32" t="s" s="2">
         <v>79</v>
@@ -4227,7 +4218,7 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>79</v>
@@ -4281,7 +4272,7 @@
         <v>194</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>73</v>
+        <v>195</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>73</v>
@@ -4302,7 +4293,7 @@
         <v>192</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH33" t="s" s="2">
         <v>79</v>
@@ -4316,10 +4307,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4327,7 +4318,7 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G34" t="s" s="2">
         <v>79</v>
@@ -4342,13 +4333,13 @@
         <v>73</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>196</v>
+        <v>152</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>196</v>
+        <v>152</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4378,10 +4369,10 @@
         <v>73</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>197</v>
+        <v>73</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>198</v>
+        <v>73</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>73</v>
@@ -4399,10 +4390,10 @@
         <v>73</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH34" t="s" s="2">
         <v>79</v>
@@ -4411,15 +4402,15 @@
         <v>73</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4427,7 +4418,7 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>79</v>
@@ -4442,13 +4433,13 @@
         <v>73</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="L35" t="s" s="2">
         <v>155</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4499,10 +4490,10 @@
         <v>73</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>199</v>
+        <v>157</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH35" t="s" s="2">
         <v>79</v>
@@ -4511,26 +4502,26 @@
         <v>73</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>73</v>
@@ -4542,15 +4533,17 @@
         <v>73</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="N36" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>163</v>
+      </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>73</v>
@@ -4587,50 +4580,50 @@
         <v>73</v>
       </c>
       <c r="AB36" t="s" s="2">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="AC36" t="s" s="2">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="AD36" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE36" t="s" s="2">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>162</v>
+        <v>73</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>73</v>
@@ -4642,16 +4635,16 @@
         <v>73</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -4689,39 +4682,39 @@
         <v>73</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>167</v>
+        <v>73</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>168</v>
+        <v>73</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>169</v>
+        <v>73</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AG37" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -4729,7 +4722,7 @@
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>79</v>
@@ -4744,17 +4737,15 @@
         <v>73</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>175</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>73</v>
@@ -4803,10 +4794,10 @@
         <v>73</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AG38" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH38" t="s" s="2">
         <v>79</v>
@@ -4815,15 +4806,15 @@
         <v>73</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>73</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -4846,13 +4837,13 @@
         <v>73</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>178</v>
+        <v>117</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -4903,7 +4894,7 @@
         <v>73</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>74</v>
@@ -4915,15 +4906,15 @@
         <v>73</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>182</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -4949,10 +4940,10 @@
         <v>117</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5003,7 +4994,7 @@
         <v>73</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>74</v>
@@ -5015,106 +5006,6 @@
         <v>73</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="B41" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="C41" s="2"/>
-      <c r="D41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="E41" s="2"/>
-      <c r="F41" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="G41" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="I41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="J41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="K41" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="L41" t="s" s="2">
-        <v>186</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>186</v>
-      </c>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="Q41" s="2"/>
-      <c r="R41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="S41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="T41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="U41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="V41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="W41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="X41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="Y41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="Z41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AA41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF41" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="AG41" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AH41" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI41" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AJ41" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>